<commit_message>
Add step 2 design values to notes
</commit_message>
<xml_diff>
--- a/WWTW_Design.xlsx
+++ b/WWTW_Design.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/A0573E005971505D/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="264" documentId="8_{D815FE4C-8060-4240-8A83-DFFA38803A91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0D8CCBC-8120-4E1C-972F-594FC0130142}"/>
+  <xr:revisionPtr revIDLastSave="311" documentId="8_{D815FE4C-8060-4240-8A83-DFFA38803A91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C28FE5BF-9C15-43E6-857F-D6DC318E9DB0}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="11700" windowHeight="11370" xr2:uid="{1B5767EC-F8E6-49E9-8072-E9EF0C9EE9E5}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="11370" windowHeight="11370" activeTab="1" xr2:uid="{1B5767EC-F8E6-49E9-8072-E9EF0C9EE9E5}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="134">
   <si>
     <t>Parameter</t>
   </si>
@@ -298,6 +298,150 @@
   </si>
   <si>
     <t>The Directive’s BOD limit is measured without nitrification, so nitrification oxygen demand is additional.</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Primary overflow rate at DWF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m³/m²/d	</t>
+  </si>
+  <si>
+    <t>Typical (range 30–50)</t>
+  </si>
+  <si>
+    <t>SNU lecture notes L14 (ocw.snu.ac.kr)</t>
+  </si>
+  <si>
+    <t>Primary overflow rate at FFT</t>
+  </si>
+  <si>
+    <t>Primary retention time at DWF</t>
+  </si>
+  <si>
+    <t>BOD removal</t>
+  </si>
+  <si>
+    <t>Within 25–40%</t>
+  </si>
+  <si>
+    <t>SNU L14; CED Engineering primary treatment text</t>
+  </si>
+  <si>
+    <t>SS removal</t>
+  </si>
+  <si>
+    <t>Within 50–65%</t>
+  </si>
+  <si>
+    <t>CED Engineering (SNU L14 gives 50–70%)</t>
+  </si>
+  <si>
+    <t>COD removal</t>
+  </si>
+  <si>
+    <t>Assumption (same as BOD)</t>
+  </si>
+  <si>
+    <t>–</t>
+  </si>
+  <si>
+    <t>TKN removal</t>
+  </si>
+  <si>
+    <t>Assumption</t>
+  </si>
+  <si>
+    <t>Ammonia-N removal</t>
+  </si>
+  <si>
+    <t>Assumption (soluble, unchanged)</t>
+  </si>
+  <si>
+    <t>Number of primary tanks</t>
+  </si>
+  <si>
+    <t>Design choice</t>
+  </si>
+  <si>
+    <t>Screen velocity through openings</t>
+  </si>
+  <si>
+    <t>m/s</t>
+  </si>
+  <si>
+    <t>Within 0.6–1.2</t>
+  </si>
+  <si>
+    <t>NPTEL Lecture 21 (screening)</t>
+  </si>
+  <si>
+    <t>Screen clear spacing</t>
+  </si>
+  <si>
+    <t>mm</t>
+  </si>
+  <si>
+    <t>Design choice (medium screens 20–50 mm)</t>
+  </si>
+  <si>
+    <t>NPTEL Lecture 21</t>
+  </si>
+  <si>
+    <t>Screen bar width</t>
+  </si>
+  <si>
+    <t>Typical (~10 mm bars)</t>
+  </si>
+  <si>
+    <t>Clean-screen headloss</t>
+  </si>
+  <si>
+    <t>0.0729(V² − v²)</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>Formula from source</t>
+  </si>
+  <si>
+    <t>Grit detention time at FFT</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>waterandwastewater.com: “30 seconds to several minutes” (page cites no source)</t>
+  </si>
+  <si>
+    <t>m³/m²/d</t>
+  </si>
+  <si>
+    <t>Typical (range 80–120)</t>
+  </si>
+  <si>
+    <t>SNU lecture notes L14</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t>Typical (range 1.5–2.5)</t>
+  </si>
+  <si>
+    <t>SNU L14; CED Engineering text gives 1.5 h before activated sludge</t>
+  </si>
+  <si>
+    <t>Step 2 criteria come mainly from US and Indian lecture and textbook material, not UK standards.</t>
   </si>
 </sst>
 </file>
@@ -305,9 +449,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="169" formatCode="#,##0.0"/>
-    <numFmt numFmtId="170" formatCode="0.000"/>
-    <numFmt numFmtId="171" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="#,##0.0"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -355,26 +499,39 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -389,6 +546,20 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E011882-5DEB-40AE-A890-C0F7596B9438}" name="Table1" displayName="Table1" ref="A8:E22" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A8:E22" xr:uid="{2E011882-5DEB-40AE-A890-C0F7596B9438}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{2CFF8964-333B-41B4-B18E-46667A53AAB1}" name="Item"/>
+    <tableColumn id="2" xr3:uid="{DC7A92A5-1FA4-4DDE-94AE-66B61981549E}" name="Value"/>
+    <tableColumn id="3" xr3:uid="{9C223776-9549-457C-A73D-AFD3B125CC0B}" name="Unit"/>
+    <tableColumn id="4" xr3:uid="{BFA6D36A-B2FF-4DF6-BCC2-32682A12449C}" name="Status"/>
+    <tableColumn id="5" xr3:uid="{97599BD9-7AB3-4E4D-8F96-F42A35E5828B}" name="Source"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1307,53 +1478,310 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4ED35503-1FDB-4344-A7E4-2522F6B534CB}">
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="100.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="43.90625" customWidth="1"/>
+    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="12" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A2" s="7"/>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A3" s="7" t="s">
+    <row r="2" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="12" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" s="7"/>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A5" s="7" t="s">
+    <row r="3" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="12" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A6" s="7"/>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A7" s="7" t="s">
+    <row r="4" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="12" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A8" s="7"/>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A9" s="7" t="s">
+    <row r="5" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="12" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A10" s="7"/>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="8"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="7"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9">
+        <v>40</v>
+      </c>
+      <c r="C9" t="s">
+        <v>90</v>
+      </c>
+      <c r="D9" t="s">
+        <v>91</v>
+      </c>
+      <c r="E9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="10">
+        <v>100</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A11" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="10">
+        <v>2</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A12" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="B12" s="10">
+        <v>30</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="B13" s="10">
+        <v>60</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="B14" s="10">
+        <v>30</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="B15" s="10">
+        <v>10</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A16" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="B16" s="10">
+        <v>0</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="B17" s="10">
+        <v>2</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="B18" s="10">
+        <v>0.9</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="B19" s="10">
+        <v>20</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="B20" s="10">
+        <v>10</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A21" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" s="10">
+        <v>180</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="11" t="s">
+        <v>133</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add step 3 parameters to notes
</commit_message>
<xml_diff>
--- a/WWTW_Design.xlsx
+++ b/WWTW_Design.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/A0573E005971505D/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="311" documentId="8_{D815FE4C-8060-4240-8A83-DFFA38803A91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C28FE5BF-9C15-43E6-857F-D6DC318E9DB0}"/>
+  <xr:revisionPtr revIDLastSave="334" documentId="8_{D815FE4C-8060-4240-8A83-DFFA38803A91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7462D4E-E517-4239-B847-5987C9315E82}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="11370" windowHeight="11370" activeTab="1" xr2:uid="{1B5767EC-F8E6-49E9-8072-E9EF0C9EE9E5}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="11700" windowHeight="11370" activeTab="1" xr2:uid="{1B5767EC-F8E6-49E9-8072-E9EF0C9EE9E5}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="193">
   <si>
     <t>Parameter</t>
   </si>
@@ -441,7 +441,240 @@
     <t>SNU L14; CED Engineering text gives 1.5 h before activated sludge</t>
   </si>
   <si>
-    <t>Step 2 criteria come mainly from US and Indian lecture and textbook material, not UK standards.</t>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Step 2:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> criteria come mainly from US and Indian lecture and textbook material, not UK standards.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Step 3:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> aeration tank parameters</t>
+    </r>
+  </si>
+  <si>
+    <t>Design temperature</t>
+  </si>
+  <si>
+    <t>Assumption (sweep 8–20 °C)</t>
+  </si>
+  <si>
+    <t>Nitrifier growth rate at 15 °C</t>
+  </si>
+  <si>
+    <t>1/d</t>
+  </si>
+  <si>
+    <t>Secondary source</t>
+  </si>
+  <si>
+    <t>US design calculation, Appendix E (vtsv.org)</t>
+  </si>
+  <si>
+    <t>Temperature correction</t>
+  </si>
+  <si>
+    <t>e^(0.098(T−15))</t>
+  </si>
+  <si>
+    <t>Same</t>
+  </si>
+  <si>
+    <t>Dissolved oxygen in tank</t>
+  </si>
+  <si>
+    <t>Secondary source (example value)</t>
+  </si>
+  <si>
+    <t>Oxygen half-saturation constant</t>
+  </si>
+  <si>
+    <t>Safety factor on minimum SRT</t>
+  </si>
+  <si>
+    <t>Secondary source (typical range 1.5–2.5)</t>
+  </si>
+  <si>
+    <t>Design effluent ammonia-N</t>
+  </si>
+  <si>
+    <t>Secondary source (example value); leaves headroom under the 5 mg/L consent</t>
+  </si>
+  <si>
+    <t>Ammonia half-saturation Kn</t>
+  </si>
+  <si>
+    <t>10^(0.051T − 1.158)</t>
+  </si>
+  <si>
+    <r>
+      <t>VERIFY:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> from memory of the standard text; consistent with the source example</t>
+    </r>
+  </si>
+  <si>
+    <t>bCOD : BOD5</t>
+  </si>
+  <si>
+    <t>g/g</t>
+  </si>
+  <si>
+    <t>Sourced</t>
+  </si>
+  <si>
+    <t>NPTEL Lecture 26 design example</t>
+  </si>
+  <si>
+    <t>Effluent soluble bCOD</t>
+  </si>
+  <si>
+    <t>Heterotroph yield</t>
+  </si>
+  <si>
+    <t>g VSS/g bCOD</t>
+  </si>
+  <si>
+    <t>Typical (range 0.4–0.6)</t>
+  </si>
+  <si>
+    <t>SNU lecture notes L18, citing Metcalf &amp; Eddy</t>
+  </si>
+  <si>
+    <t>Decay coefficient at 20 °C</t>
+  </si>
+  <si>
+    <t>Typical (range 0.06–0.15)</t>
+  </si>
+  <si>
+    <t>SNU L18</t>
+  </si>
+  <si>
+    <t>Decay temperature coefficient</t>
+  </si>
+  <si>
+    <r>
+      <t>VERIFY:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> from memory; the source gives only a generic 1.02–1.25 range</t>
+    </r>
+  </si>
+  <si>
+    <t>SNU L18 (range only)</t>
+  </si>
+  <si>
+    <t>Cell debris fraction</t>
+  </si>
+  <si>
+    <t>Typical (range 0.10–0.15)</t>
+  </si>
+  <si>
+    <t>Biomass VSS/TSS</t>
+  </si>
+  <si>
+    <t>Typical</t>
+  </si>
+  <si>
+    <t>SNU L19</t>
+  </si>
+  <si>
+    <t>MLSS</t>
+  </si>
+  <si>
+    <t>Top of the 1,500–4,000 complete-mix range</t>
+  </si>
+  <si>
+    <t>MIT 1.85 lecture notes (L20)</t>
+  </si>
+  <si>
+    <t>MLVSS : MLSS</t>
+  </si>
+  <si>
+    <t>Inert fraction of incoming SS</t>
+  </si>
+  <si>
+    <t>Nitrogen content of biomass</t>
+  </si>
+  <si>
+    <t>g N/g VSS</t>
+  </si>
+  <si>
+    <t>Calculated from C₅H₇O₂N (14 ÷ 113)</t>
+  </si>
+  <si>
+    <t>Oxygen per g biomass produced</t>
+  </si>
+  <si>
+    <t>Oxygen per g NH₄-N oxidised</t>
+  </si>
+  <si>
+    <t>NPTEL Lecture 26</t>
+  </si>
+  <si>
+    <t>Alkalinity used per g NH₄-N oxidised</t>
+  </si>
+  <si>
+    <t>g CaCO₃/g</t>
+  </si>
+  <si>
+    <t>Calculated from the reaction stoichiometry</t>
+  </si>
+  <si>
+    <t>Nitrifier biomass growth and nitrite are ignored.</t>
+  </si>
+  <si>
+    <t>Soluble organic nitrogen in the effluent is ignored.</t>
+  </si>
+  <si>
+    <t>There is no anoxic zone, so no denitrification credit.</t>
+  </si>
+  <si>
+    <t>Kn and the decay temperature coefficient are from memory of the standard text and still to be verified.</t>
+  </si>
+  <si>
+    <t>Alkalinity supply is not in the design basis, so adequacy is not checked.</t>
   </si>
 </sst>
 </file>
@@ -499,7 +732,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -518,16 +751,37 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="5">
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -549,7 +803,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E011882-5DEB-40AE-A890-C0F7596B9438}" name="Table1" displayName="Table1" ref="A8:E22" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E011882-5DEB-40AE-A890-C0F7596B9438}" name="Table1" displayName="Table1" ref="A8:E22" totalsRowShown="0" headerRowDxfId="4">
   <autoFilter ref="A8:E22" xr:uid="{2E011882-5DEB-40AE-A890-C0F7596B9438}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{2CFF8964-333B-41B4-B18E-46667A53AAB1}" name="Item"/>
@@ -557,6 +811,20 @@
     <tableColumn id="3" xr3:uid="{9C223776-9549-457C-A73D-AFD3B125CC0B}" name="Unit"/>
     <tableColumn id="4" xr3:uid="{BFA6D36A-B2FF-4DF6-BCC2-32682A12449C}" name="Status"/>
     <tableColumn id="5" xr3:uid="{97599BD9-7AB3-4E4D-8F96-F42A35E5828B}" name="Source"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{10220E0A-F588-4EEC-850B-7E1E2D028A41}" name="Table2" displayName="Table2" ref="A25:E47" totalsRowShown="0">
+  <autoFilter ref="A25:E47" xr:uid="{10220E0A-F588-4EEC-850B-7E1E2D028A41}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{A1F7691C-638B-4B2A-B87A-F15E20AFA8EB}" name="Item"/>
+    <tableColumn id="2" xr3:uid="{1CD2E7D3-4A29-4294-A4B7-8E9D80737189}" name="Value" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{DA10D8A3-F7B5-4974-AEA0-6F8A2B592C26}" name="Unit" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{04AE792B-44D8-48DF-B396-C0B22157B224}" name="Status" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{9D8EB251-4103-49AC-B5D7-844043A24FDC}" name="Source" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1478,45 +1746,47 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4ED35503-1FDB-4344-A7E4-2522F6B534CB}">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="43.90625" customWidth="1"/>
-    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.26953125" customWidth="1"/>
     <col min="4" max="4" width="20.453125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="32.36328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="11" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="11" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="11" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="11" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="11" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="8"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="7"/>
+    <row r="7" spans="1:5" s="8" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="11" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
@@ -1705,7 +1975,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="10" t="s">
         <v>114</v>
       </c>
@@ -1773,15 +2043,442 @@
         <v>126</v>
       </c>
     </row>
-    <row r="24" spans="1:5" s="11" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="11" t="s">
-        <v>133</v>
-      </c>
+    <row r="24" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="12" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A26" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B26" s="10">
+        <v>10</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D26" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="E26" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A27" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="B27" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="D27" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A28" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D28" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E28" s="10" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A29" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="B29" s="10">
+        <v>2</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D29" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="B30" s="10">
+        <v>1.3</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D30" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E30" s="10" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A31" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B31" s="10">
+        <v>2</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="E31" s="10" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A32" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="B32" s="10">
+        <v>1</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D32" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="E32" s="10" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A33" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="C33" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="E33" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="B34" s="10">
+        <v>1.47</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="E34" s="10" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A35" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="B35" s="10">
+        <v>5</v>
+      </c>
+      <c r="C35" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E35" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A36" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="B36" s="10">
+        <v>0.45</v>
+      </c>
+      <c r="C36" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="E36" s="10" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A37" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="B37" s="10">
+        <v>0.1</v>
+      </c>
+      <c r="C37" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="E37" s="10" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A38" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="B38" s="10">
+        <v>1.04</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="E38" s="10" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A39" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="B39" s="10">
+        <v>0.15</v>
+      </c>
+      <c r="C39" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A40" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="B40" s="10">
+        <v>0.85</v>
+      </c>
+      <c r="C40" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D40" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="E40" s="10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A41" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="B41" s="15">
+        <v>4000</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D41" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="E41" s="10" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A42" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="B42" s="10">
+        <v>0.75</v>
+      </c>
+      <c r="C42" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D42" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E42" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A43" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="B43" s="10">
+        <v>0.4</v>
+      </c>
+      <c r="C43" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D43" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E43" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A44" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="B44" s="10">
+        <v>0.124</v>
+      </c>
+      <c r="C44" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="D44" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="E44" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A45" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="B45" s="10">
+        <v>1.42</v>
+      </c>
+      <c r="C45" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="D45" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="E45" s="10" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A46" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="B46" s="10">
+        <v>4.33</v>
+      </c>
+      <c r="C46" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="D46" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="E46" s="10" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A47" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="B47" s="10">
+        <v>7.14</v>
+      </c>
+      <c r="C47" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="D47" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="E47" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A49" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="B49" s="7"/>
+      <c r="C49" s="7"/>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A50" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="B50" s="7"/>
+      <c r="C50" s="7"/>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A51" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="B51" s="7"/>
+      <c r="C51" s="7"/>
+    </row>
+    <row r="52" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A52" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="B52" s="7"/>
+      <c r="C52" s="7"/>
+    </row>
+    <row r="53" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A53" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="B53" s="7"/>
+      <c r="C53" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
+  <tableParts count="2">
     <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add step 4 parameters to notes
</commit_message>
<xml_diff>
--- a/WWTW_Design.xlsx
+++ b/WWTW_Design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/A0573E005971505D/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="334" documentId="8_{D815FE4C-8060-4240-8A83-DFFA38803A91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7462D4E-E517-4239-B847-5987C9315E82}"/>
+  <xr:revisionPtr revIDLastSave="348" documentId="8_{D815FE4C-8060-4240-8A83-DFFA38803A91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D900707-2EF9-4E4C-85B1-BE4B6CC5AB9B}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="0" windowWidth="11700" windowHeight="11370" activeTab="1" xr2:uid="{1B5767EC-F8E6-49E9-8072-E9EF0C9EE9E5}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="231">
   <si>
     <t>Parameter</t>
   </si>
@@ -439,44 +439,6 @@
   </si>
   <si>
     <t>SNU L14; CED Engineering text gives 1.5 h before activated sludge</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Step 2:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> criteria come mainly from US and Indian lecture and textbook material, not UK standards.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Step 3:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> aeration tank parameters</t>
-    </r>
   </si>
   <si>
     <t>Design temperature</t>
@@ -675,6 +637,139 @@
   </si>
   <si>
     <t>Alkalinity supply is not in the design basis, so adequacy is not checked.</t>
+  </si>
+  <si>
+    <t>Step 4: secondary clarifier parameters</t>
+  </si>
+  <si>
+    <t>Step 3: aeration tank parameters</t>
+  </si>
+  <si>
+    <t>Step 2: criteria come mainly from US and Indian lecture and textbook material, not UK standards.</t>
+  </si>
+  <si>
+    <t>Design SVI</t>
+  </si>
+  <si>
+    <t>mL/g</t>
+  </si>
+  <si>
+    <t>Design choice within the typical 75–150 range</t>
+  </si>
+  <si>
+    <t>Iowa State course notes (Activated Sludge Design Equations)</t>
+  </si>
+  <si>
+    <t>Return sludge concentration</t>
+  </si>
+  <si>
+    <t>10⁶ ÷ SVI</t>
+  </si>
+  <si>
+    <t>Sourced relationship</t>
+  </si>
+  <si>
+    <t>Return ratio</t>
+  </si>
+  <si>
+    <t>MLSS ÷ (Xr − MLSS)</t>
+  </si>
+  <si>
+    <t>Mass balance</t>
+  </si>
+  <si>
+    <t>Surface overflow rate, average flow</t>
+  </si>
+  <si>
+    <t>One plant’s design basis, not a standard</t>
+  </si>
+  <si>
+    <t>Winnipeg SEWPCC conceptual design report</t>
+  </si>
+  <si>
+    <t>Surface overflow rate, peak flow</t>
+  </si>
+  <si>
+    <t>Same; applied to our FFT, which is conservative</t>
+  </si>
+  <si>
+    <t>Solids loading rate, average flow</t>
+  </si>
+  <si>
+    <t>kg/m²/d</t>
+  </si>
+  <si>
+    <t>Solids loading rate, peak flow</t>
+  </si>
+  <si>
+    <t>Weir loading limit</t>
+  </si>
+  <si>
+    <t>m³/m/d</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Plants over 1 mgd; source table hard to read, so </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>verify</t>
+    </r>
+  </si>
+  <si>
+    <t>Iowa State course notes</t>
+  </si>
+  <si>
+    <t>Number of clarifiers</t>
+  </si>
+  <si>
+    <t>Design choice (two or more, circular)</t>
+  </si>
+  <si>
+    <t>Iowa State design notes</t>
+  </si>
+  <si>
+    <t>Side water depth</t>
+  </si>
+  <si>
+    <t>Assumption (the Winnipeg report uses 4.6 m)</t>
+  </si>
+  <si>
+    <t>Return flow at FFT</t>
+  </si>
+  <si>
+    <t>held at the DWF-based value</t>
+  </si>
+  <si>
+    <t>Tank diameter rounding</t>
+  </si>
+  <si>
+    <t>up to the next 0.5</t>
+  </si>
+  <si>
+    <t>Criteria come from one existing plant’s design basis and lecture notes, not a standard; UK practice not checked.</t>
+  </si>
+  <si>
+    <t>The peak overflow rate comes from a maximum-week flow but is applied to the FFT.</t>
+  </si>
+  <si>
+    <t>MLSS held at 4,000 mg/L and the return flow held constant at peak flow.</t>
+  </si>
+  <si>
+    <t>Effluent solids loss is not included in the sludge age.</t>
+  </si>
+  <si>
+    <t>Weir length assumes a weir on the tank edge only; no sludge blanket or flux (state point) analysis.</t>
+  </si>
+  <si>
+    <t>The tanks work only up to an SVI of about 105 mL/g; a bulking sludge needs more area.</t>
   </si>
 </sst>
 </file>
@@ -732,7 +827,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -765,11 +860,26 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="9">
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -803,7 +913,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E011882-5DEB-40AE-A890-C0F7596B9438}" name="Table1" displayName="Table1" ref="A8:E22" totalsRowShown="0" headerRowDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E011882-5DEB-40AE-A890-C0F7596B9438}" name="Table1" displayName="Table1" ref="A8:E22" totalsRowShown="0" headerRowDxfId="8">
   <autoFilter ref="A8:E22" xr:uid="{2E011882-5DEB-40AE-A890-C0F7596B9438}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{2CFF8964-333B-41B4-B18E-46667A53AAB1}" name="Item"/>
@@ -821,10 +931,24 @@
   <autoFilter ref="A25:E47" xr:uid="{10220E0A-F588-4EEC-850B-7E1E2D028A41}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{A1F7691C-638B-4B2A-B87A-F15E20AFA8EB}" name="Item"/>
-    <tableColumn id="2" xr3:uid="{1CD2E7D3-4A29-4294-A4B7-8E9D80737189}" name="Value" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{DA10D8A3-F7B5-4974-AEA0-6F8A2B592C26}" name="Unit" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{04AE792B-44D8-48DF-B396-C0B22157B224}" name="Status" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{9D8EB251-4103-49AC-B5D7-844043A24FDC}" name="Source" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{1CD2E7D3-4A29-4294-A4B7-8E9D80737189}" name="Value" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{DA10D8A3-F7B5-4974-AEA0-6F8A2B592C26}" name="Unit" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{04AE792B-44D8-48DF-B396-C0B22157B224}" name="Status" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{9D8EB251-4103-49AC-B5D7-844043A24FDC}" name="Source" dataDxfId="4"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B6766CDA-76F9-4B7B-9856-32898855FE7B}" name="Table3" displayName="Table3" ref="A56:E68" totalsRowShown="0">
+  <autoFilter ref="A56:E68" xr:uid="{B6766CDA-76F9-4B7B-9856-32898855FE7B}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{E0CFC413-A1FA-4747-9B82-F17D183B11D4}" name="Item"/>
+    <tableColumn id="2" xr3:uid="{55FA7182-7794-4DEB-86DE-BEEF2880D08B}" name="Value" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{B12F1A64-7555-463C-B711-5C7C438C3C74}" name="Unit" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{258BFD5C-E2FB-4A9A-BF30-E43CE2E1A031}" name="Status" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{84CE2C52-D72B-470E-8872-B014E10B2DDE}" name="Source" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1746,7 +1870,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4ED35503-1FDB-4344-A7E4-2522F6B534CB}">
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="43.90625" customWidth="1"/>
@@ -1784,8 +1908,8 @@
       <c r="A6" s="8"/>
     </row>
     <row r="7" spans="1:5" s="8" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="11" t="s">
-        <v>133</v>
+      <c r="A7" s="16" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -2045,7 +2169,7 @@
     </row>
     <row r="24" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" s="12" t="s">
-        <v>134</v>
+        <v>192</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
@@ -2067,7 +2191,7 @@
     </row>
     <row r="26" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="10" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B26" s="10">
         <v>10</v>
@@ -2076,7 +2200,7 @@
         <v>74</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E26" s="10" t="s">
         <v>103</v>
@@ -2084,41 +2208,41 @@
     </row>
     <row r="27" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B27" s="10">
         <v>0.5</v>
       </c>
       <c r="C27" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="D27" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="E27" s="10" t="s">
         <v>138</v>
-      </c>
-      <c r="D27" s="10" t="s">
-        <v>139</v>
-      </c>
-      <c r="E27" s="10" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="10" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C28" s="10" t="s">
         <v>103</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A29" s="10" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B29" s="10">
         <v>2</v>
@@ -2127,15 +2251,15 @@
         <v>75</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="10" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B30" s="10">
         <v>1.3</v>
@@ -2144,15 +2268,15 @@
         <v>75</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A31" s="10" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B31" s="10">
         <v>2</v>
@@ -2161,15 +2285,15 @@
         <v>103</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="58" x14ac:dyDescent="0.35">
       <c r="A32" s="10" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B32" s="10">
         <v>1</v>
@@ -2178,24 +2302,24 @@
         <v>75</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="58" x14ac:dyDescent="0.35">
       <c r="A33" s="10" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C33" s="10" t="s">
         <v>75</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E33" s="10" t="s">
         <v>103</v>
@@ -2203,24 +2327,24 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="10" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B34" s="10">
         <v>1.47</v>
       </c>
       <c r="C34" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="E34" s="10" t="s">
         <v>155</v>
-      </c>
-      <c r="D34" s="10" t="s">
-        <v>156</v>
-      </c>
-      <c r="E34" s="10" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B35" s="10">
         <v>5</v>
@@ -2237,41 +2361,41 @@
     </row>
     <row r="36" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A36" s="10" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B36" s="10">
         <v>0.45</v>
       </c>
       <c r="C36" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="E36" s="10" t="s">
         <v>160</v>
-      </c>
-      <c r="D36" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="E36" s="10" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A37" s="10" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B37" s="10">
         <v>0.1</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A38" s="10" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B38" s="10">
         <v>1.04</v>
@@ -2280,15 +2404,15 @@
         <v>103</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A39" s="10" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B39" s="10">
         <v>0.15</v>
@@ -2297,15 +2421,15 @@
         <v>103</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="10" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B40" s="10">
         <v>0.85</v>
@@ -2314,15 +2438,15 @@
         <v>103</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A41" s="10" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B41" s="15">
         <v>4000</v>
@@ -2331,15 +2455,15 @@
         <v>75</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="10" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B42" s="10">
         <v>0.75</v>
@@ -2356,7 +2480,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="10" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B43" s="10">
         <v>0.4</v>
@@ -2373,16 +2497,16 @@
     </row>
     <row r="44" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A44" s="10" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B44" s="10">
         <v>0.124</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="E44" s="10" t="s">
         <v>103</v>
@@ -2390,95 +2514,370 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="10" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B45" s="10">
         <v>1.42</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="10" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B46" s="10">
         <v>4.33</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A47" s="10" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B47" s="10">
         <v>7.14</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="E47" s="10" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="7" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B49" s="7"/>
       <c r="C49" s="7"/>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="7" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B50" s="7"/>
       <c r="C50" s="7"/>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="7" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B51" s="7"/>
       <c r="C51" s="7"/>
     </row>
-    <row r="52" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A52" s="7" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B52" s="7"/>
       <c r="C52" s="7"/>
     </row>
-    <row r="53" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A53" s="7" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B53" s="7"/>
       <c r="C53" s="7"/>
     </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A55" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A56" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="B56" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C56" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D56" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="E56" s="13" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A57" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="B57" s="10">
+        <v>100</v>
+      </c>
+      <c r="C57" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="D57" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="E57" s="10" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A58" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="B58" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="C58" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D58" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="E58" s="10" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A59" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="B59" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="C59" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D59" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="E59" s="10" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A60" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="B60" s="10">
+        <v>24</v>
+      </c>
+      <c r="C60" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="D60" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="E60" s="10" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A61" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="B61" s="10">
+        <v>44</v>
+      </c>
+      <c r="C61" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="D61" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="E61" s="10" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A62" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="B62" s="10">
+        <v>144</v>
+      </c>
+      <c r="C62" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="D62" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="E62" s="10" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A63" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B63" s="10">
+        <v>216</v>
+      </c>
+      <c r="C63" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="D63" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="E63" s="10" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A64" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="B64" s="10">
+        <v>375</v>
+      </c>
+      <c r="C64" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="D64" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="E64" s="10" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A65" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="B65" s="10">
+        <v>2</v>
+      </c>
+      <c r="C65" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D65" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="E65" s="10" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A66" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="B66" s="10">
+        <v>4</v>
+      </c>
+      <c r="C66" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="D66" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="E66" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A67" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="B67" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="C67" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D67" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E67" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A68" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="B68" s="10" t="s">
+        <v>224</v>
+      </c>
+      <c r="C68" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="D68" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="E68" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A70" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="B70" s="7"/>
+      <c r="C70" s="7"/>
+      <c r="D70" s="7"/>
+    </row>
+    <row r="71" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A71" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="B71" s="7"/>
+      <c r="C71" s="7"/>
+      <c r="D71" s="7"/>
+    </row>
+    <row r="72" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A72" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="B72" s="7"/>
+      <c r="C72" s="7"/>
+      <c r="D72" s="7"/>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A73" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="B73" s="7"/>
+      <c r="C73" s="7"/>
+      <c r="D73" s="7"/>
+    </row>
+    <row r="74" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A74" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="B74" s="7"/>
+      <c r="C74" s="7"/>
+      <c r="D74" s="7"/>
+    </row>
+    <row r="75" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A75" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="B75" s="7"/>
+      <c r="C75" s="7"/>
+      <c r="D75" s="7"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="2">
+  <tableParts count="3">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update workbook: trim sources, add Sources sheet
</commit_message>
<xml_diff>
--- a/WWTW_Design.xlsx
+++ b/WWTW_Design.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/A0573E005971505D/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="348" documentId="8_{D815FE4C-8060-4240-8A83-DFFA38803A91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D900707-2EF9-4E4C-85B1-BE4B6CC5AB9B}"/>
+  <xr:revisionPtr revIDLastSave="443" documentId="8_{D815FE4C-8060-4240-8A83-DFFA38803A91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6768CEBC-ACD2-4EA7-8DCC-FD13C6ACED18}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="0" windowWidth="11700" windowHeight="11370" activeTab="1" xr2:uid="{1B5767EC-F8E6-49E9-8072-E9EF0C9EE9E5}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
     <sheet name="Notes" sheetId="2" r:id="rId2"/>
+    <sheet name="Sources" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="299">
   <si>
     <t>Parameter</t>
   </si>
@@ -156,12 +157,6 @@
     <t>Secondary source: same</t>
   </si>
   <si>
-    <t>Weak source: lecture notes, typical 5.4-5.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Xylem: 1.8-2.2 typical </t>
-  </si>
-  <si>
     <t>SEPA: FFT = 3PG + Imax + 3E</t>
   </si>
   <si>
@@ -177,9 +172,6 @@
     <t>Directive Annex I Table 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Directive Annex I Table of </t>
-  </si>
-  <si>
     <t>Directive Annex I Table 1 (over 10,000 p.e.)</t>
   </si>
   <si>
@@ -291,9 +283,6 @@
     <t>Infiltration, trade effluent, temperatures and the ammonia consent are assumptions.</t>
   </si>
   <si>
-    <t>SS and ammonia loads come from a secondary source (WTI 1994 via Peiris, WEDC); organic N comes from lecture notes.</t>
-  </si>
-  <si>
     <t>Consent limits are treated as upper limits, which is conservative, since the Directive allows a set number of failed samples.</t>
   </si>
   <si>
@@ -315,12 +304,6 @@
     <t xml:space="preserve">m³/m²/d	</t>
   </si>
   <si>
-    <t>Typical (range 30–50)</t>
-  </si>
-  <si>
-    <t>SNU lecture notes L14 (ocw.snu.ac.kr)</t>
-  </si>
-  <si>
     <t>Primary overflow rate at FFT</t>
   </si>
   <si>
@@ -330,21 +313,9 @@
     <t>BOD removal</t>
   </si>
   <si>
-    <t>Within 25–40%</t>
-  </si>
-  <si>
-    <t>SNU L14; CED Engineering primary treatment text</t>
-  </si>
-  <si>
     <t>SS removal</t>
   </si>
   <si>
-    <t>Within 50–65%</t>
-  </si>
-  <si>
-    <t>CED Engineering (SNU L14 gives 50–70%)</t>
-  </si>
-  <si>
     <t>COD removal</t>
   </si>
   <si>
@@ -420,27 +391,12 @@
     <t>s</t>
   </si>
   <si>
-    <t>waterandwastewater.com: “30 seconds to several minutes” (page cites no source)</t>
-  </si>
-  <si>
     <t>m³/m²/d</t>
   </si>
   <si>
-    <t>Typical (range 80–120)</t>
-  </si>
-  <si>
-    <t>SNU lecture notes L14</t>
-  </si>
-  <si>
     <t>h</t>
   </si>
   <si>
-    <t>Typical (range 1.5–2.5)</t>
-  </si>
-  <si>
-    <t>SNU L14; CED Engineering text gives 1.5 h before activated sludge</t>
-  </si>
-  <si>
     <t>Design temperature</t>
   </si>
   <si>
@@ -493,21 +449,6 @@
   </si>
   <si>
     <t>10^(0.051T − 1.158)</t>
-  </si>
-  <si>
-    <r>
-      <t>VERIFY:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> from memory of the standard text; consistent with the source example</t>
-    </r>
   </si>
   <si>
     <t>bCOD : BOD5</t>
@@ -576,12 +517,6 @@
     <t>Biomass VSS/TSS</t>
   </si>
   <si>
-    <t>Typical</t>
-  </si>
-  <si>
-    <t>SNU L19</t>
-  </si>
-  <si>
     <t>MLSS</t>
   </si>
   <si>
@@ -633,9 +568,6 @@
     <t>There is no anoxic zone, so no denitrification credit.</t>
   </si>
   <si>
-    <t>Kn and the decay temperature coefficient are from memory of the standard text and still to be verified.</t>
-  </si>
-  <si>
     <t>Alkalinity supply is not in the design basis, so adequacy is not checked.</t>
   </si>
   <si>
@@ -654,21 +586,12 @@
     <t>mL/g</t>
   </si>
   <si>
-    <t>Design choice within the typical 75–150 range</t>
-  </si>
-  <si>
-    <t>Iowa State course notes (Activated Sludge Design Equations)</t>
-  </si>
-  <si>
     <t>Return sludge concentration</t>
   </si>
   <si>
     <t>10⁶ ÷ SVI</t>
   </si>
   <si>
-    <t>Sourced relationship</t>
-  </si>
-  <si>
     <t>Return ratio</t>
   </si>
   <si>
@@ -708,8 +631,83 @@
     <t>m³/m/d</t>
   </si>
   <si>
+    <t>Number of clarifiers</t>
+  </si>
+  <si>
+    <t>Design choice (two or more, circular)</t>
+  </si>
+  <si>
+    <t>Side water depth</t>
+  </si>
+  <si>
+    <t>Assumption (the Winnipeg report uses 4.6 m)</t>
+  </si>
+  <si>
+    <t>Return flow at FFT</t>
+  </si>
+  <si>
+    <t>held at the DWF-based value</t>
+  </si>
+  <si>
+    <t>Tank diameter rounding</t>
+  </si>
+  <si>
+    <t>up to the next 0.5</t>
+  </si>
+  <si>
+    <t>Criteria come from one existing plant’s design basis and lecture notes, not a standard; UK practice not checked.</t>
+  </si>
+  <si>
+    <t>The peak overflow rate comes from a maximum-week flow but is applied to the FFT.</t>
+  </si>
+  <si>
+    <t>MLSS held at 4,000 mg/L and the return flow held constant at peak flow.</t>
+  </si>
+  <si>
+    <t>Effluent solids loss is not included in the sludge age.</t>
+  </si>
+  <si>
+    <t>Weir length assumes a weir on the tank edge only; no sludge blanket or flux (state point) analysis.</t>
+  </si>
+  <si>
+    <t>The tanks work only up to an SVI of about 105 mL/g; a bulking sludge needs more area.</t>
+  </si>
+  <si>
+    <t>5: air supply and energy parameters</t>
+  </si>
+  <si>
+    <t>Aeration tank side water depth</t>
+  </si>
+  <si>
+    <t>Diffuser height above floor</t>
+  </si>
+  <si>
+    <t>Assumption (the ORNL example uses 0.46 m)</t>
+  </si>
+  <si>
+    <t>Standard oxygen transfer efficiency</t>
+  </si>
+  <si>
+    <t>% per m submergence</t>
+  </si>
+  <si>
+    <t>Typical for fine-bubble diffusers; software documentation, not a textbook</t>
+  </si>
+  <si>
+    <t>aquakin documentation</t>
+  </si>
+  <si>
+    <t>Diffuser fouling factor</t>
+  </si>
+  <si>
+    <t>Assumption (aquakin default is 1.0)</t>
+  </si>
+  <si>
+    <t>Alpha factor</t>
+  </si>
+  <si>
     <r>
-      <t xml:space="preserve">Plants over 1 mgd; source table hard to read, so </t>
+      <t xml:space="preserve">Bottom of the 0.80–0.90 range; </t>
     </r>
     <r>
       <rPr>
@@ -722,54 +720,259 @@
       </rPr>
       <t>verify</t>
     </r>
-  </si>
-  <si>
-    <t>Iowa State course notes</t>
-  </si>
-  <si>
-    <t>Number of clarifiers</t>
-  </si>
-  <si>
-    <t>Design choice (two or more, circular)</t>
-  </si>
-  <si>
-    <t>Iowa State design notes</t>
-  </si>
-  <si>
-    <t>Side water depth</t>
-  </si>
-  <si>
-    <t>Assumption (the Winnipeg report uses 4.6 m)</t>
-  </si>
-  <si>
-    <t>Return flow at FFT</t>
-  </si>
-  <si>
-    <t>held at the DWF-based value</t>
-  </si>
-  <si>
-    <t>Tank diameter rounding</t>
-  </si>
-  <si>
-    <t>up to the next 0.5</t>
-  </si>
-  <si>
-    <t>Criteria come from one existing plant’s design basis and lecture notes, not a standard; UK practice not checked.</t>
-  </si>
-  <si>
-    <t>The peak overflow rate comes from a maximum-week flow but is applied to the FFT.</t>
-  </si>
-  <si>
-    <t>MLSS held at 4,000 mg/L and the return flow held constant at peak flow.</t>
-  </si>
-  <si>
-    <t>Effluent solids loss is not included in the sludge age.</t>
-  </si>
-  <si>
-    <t>Weir length assumes a weir on the tank edge only; no sludge blanket or flux (state point) analysis.</t>
-  </si>
-  <si>
-    <t>The tanks work only up to an SVI of about 105 mL/g; a bulking sludge needs more area.</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, because fine-bubble alpha is often lower in practice</t>
+    </r>
+  </si>
+  <si>
+    <t>ORNL aeration systems training material</t>
+  </si>
+  <si>
+    <t>Beta factor</t>
+  </si>
+  <si>
+    <t>ORNL</t>
+  </si>
+  <si>
+    <t>Oxygen saturation at 10 °C / reference at 20 °C</t>
+  </si>
+  <si>
+    <t>11.33 / 9.2</t>
+  </si>
+  <si>
+    <t>Sourced (worked example)</t>
+  </si>
+  <si>
+    <t>1.024^(T−20)</t>
+  </si>
+  <si>
+    <t>From step 3</t>
+  </si>
+  <si>
+    <t>Oxygen in standard air</t>
+  </si>
+  <si>
+    <t>kg O₂/m³</t>
+  </si>
+  <si>
+    <t>Sourced (1.204 kg/m³ × 0.2318)</t>
+  </si>
+  <si>
+    <t>Ratio of specific heats for air</t>
+  </si>
+  <si>
+    <t>Blower wire-to-air efficiency</t>
+  </si>
+  <si>
+    <t>Sourced default</t>
+  </si>
+  <si>
+    <t>Diffuser and pipework losses</t>
+  </si>
+  <si>
+    <t>kPa</t>
+  </si>
+  <si>
+    <t>Operating hours</t>
+  </si>
+  <si>
+    <t>h/year</t>
+  </si>
+  <si>
+    <t>Assumption (continuous at design load)</t>
+  </si>
+  <si>
+    <t>Aeration share of plant energy</t>
+  </si>
+  <si>
+    <t>25–60</t>
+  </si>
+  <si>
+    <t>Plant energy benchmark</t>
+  </si>
+  <si>
+    <t>28–86</t>
+  </si>
+  <si>
+    <t>kWh/PE/year</t>
+  </si>
+  <si>
+    <t>de Haas et al. (2018), Water e-Journal</t>
+  </si>
+  <si>
+    <t>Average load only; installed blower capacity needs a peaking factor that is not included.</t>
+  </si>
+  <si>
+    <t>Continuous operation at the design load for the whole year.</t>
+  </si>
+  <si>
+    <t>Standard-condition air flow; no correction for colder winter inlet air.</t>
+  </si>
+  <si>
+    <t>Transfer efficiency, fouling, pipework loss and blower efficiency are typical values from non-textbook sources, not supplier data.</t>
+  </si>
+  <si>
+    <t>No energy for mixing, pumping, return sludge or sludge treatment; no denitrification credit.</t>
+  </si>
+  <si>
+    <t>Assumption (typical value; ammonia 8 + organic 5 = TKN 13 g N/head/d)</t>
+  </si>
+  <si>
+    <t>Assumption (typical value)</t>
+  </si>
+  <si>
+    <t>SS and ammonia loads come from a secondary source (WTI 1994 via Peiris, WEDC); organic N is an assumption.</t>
+  </si>
+  <si>
+    <t>Assumption (typical)</t>
+  </si>
+  <si>
+    <t>Assumption (typical limit)</t>
+  </si>
+  <si>
+    <t>Benchmark is Australian data, not UK</t>
+  </si>
+  <si>
+    <t>No.</t>
+  </si>
+  <si>
+    <t>Used for</t>
+  </si>
+  <si>
+    <t>Directive 91/271/EEC, Annex I and Article 2 (legislation.gov.uk)</t>
+  </si>
+  <si>
+    <t>60 g BOD5 per PE, BOD, COD and SS consents</t>
+  </si>
+  <si>
+    <t>SEPA guidance wat-sg-13dec24</t>
+  </si>
+  <si>
+    <t>DWF and FFT formulas, 150 L/head/d</t>
+  </si>
+  <si>
+    <t>Peiris, WEDC paper, citing WTI 1994</t>
+  </si>
+  <si>
+    <t>SS 75 and ammonia-N 8 g/head/d</t>
+  </si>
+  <si>
+    <t>SNU lecture notes L18</t>
+  </si>
+  <si>
+    <t>Yield, decay, cell debris, 1.42 g O₂/g biomass</t>
+  </si>
+  <si>
+    <t>Screen velocity, spacing, headloss formula</t>
+  </si>
+  <si>
+    <t>MIT 1.85 lecture notes, L20</t>
+  </si>
+  <si>
+    <t>MLSS range</t>
+  </si>
+  <si>
+    <t>Clarifier overflow and solids loading rates</t>
+  </si>
+  <si>
+    <t>Nitrifier kinetics, safety factor</t>
+  </si>
+  <si>
+    <t>Alpha, beta, saturation values, efficiency range, aeration share</t>
+  </si>
+  <si>
+    <t>Transfer efficiency, oxygen in air, blower efficiency</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>https://legislation.gov.uk/eudr/1991/271/2020-12-31/data.html</t>
+  </si>
+  <si>
+    <t>https://sepa.org.uk/media/hkedns5b/wat-sg-13dec24.docx</t>
+  </si>
+  <si>
+    <t>https://wedc-knowledge.lboro.ac.uk/resources/conference/20/Peiris.pdf</t>
+  </si>
+  <si>
+    <t>https://ocw.snu.ac.kr/sites/default/files/NOTE/10649.pdf</t>
+  </si>
+  <si>
+    <t>https://ocw.snu.ac.kr/sites/default/files/NOTE/L18_Fundamentals%20of%20biological%20treatment%20II.pdf</t>
+  </si>
+  <si>
+    <t>https://archive.nptel.ac.in/content/storage2/courses/105104102/Lecture%2021.htm</t>
+  </si>
+  <si>
+    <t>https://archive.nptel.ac.in/content/storage2/courses/105104102/Lecture%2026.htm</t>
+  </si>
+  <si>
+    <t>https://ocw.mit.edu/courses/1-85-water-and-wastewater-treatment-engineering-spring-2006/resources/l20_acti_slud_2</t>
+  </si>
+  <si>
+    <t>https://legacy.winnipeg.ca/finance/findata/matmgt/documents/2012/682-2012/682-2012_Appendix_G-SEWPCC_Upgradin_Expansion_Conceptual_Design_Report/Sec_10_SecondClar_Jun0109.pdf</t>
+  </si>
+  <si>
+    <t>https://www.vtsv.org/wp-content/uploads/2016/05/Appendix-E-Preliminary-calculation.pdf</t>
+  </si>
+  <si>
+    <t>https://bptraining.ornl.gov/wp-content/uploads/2021/09/11-Aeration-Systems.pdf</t>
+  </si>
+  <si>
+    <t>https://aquakin.readthedocs.io/en/latest/generated/aquakin.AerationSystem.html</t>
+  </si>
+  <si>
+    <t>https://www.awa.asn.au/hubfs/Water%20e-journal/2018/May%202018/201805_003_002_023_Benchmarking%20Energy%20Use%20for%20Wastewater%20Treatment%20Plants.pdf</t>
+  </si>
+  <si>
+    <t>Typical (~2 h)</t>
+  </si>
+  <si>
+    <t>SNU slides, file 10649 (ocw.snu.ac.kr)</t>
+  </si>
+  <si>
+    <t>Source gives ~35%; 30% is slightly conservative</t>
+  </si>
+  <si>
+    <t>SNU slides, file 10649</t>
+  </si>
+  <si>
+    <t>Source gives ~60%</t>
+  </si>
+  <si>
+    <t>Secondary source (empirical formula in the example sheet)</t>
+  </si>
+  <si>
+    <t>Sourced as BODu/BOD5 (1.47); used here as a proxy for bCOD/BOD5</t>
+  </si>
+  <si>
+    <t>The decay temperature coefficient is from memory of the standard text and still to be verified.</t>
+  </si>
+  <si>
+    <t>Definition (SVI is mL settled per g solids, so Xr ≈ 10⁶ ÷ SVI)</t>
+  </si>
+  <si>
+    <t>28 = best-practice target; 86 = observed average of 245 Australian plants (2015–16); typical guide value 44. Not UK data.</t>
+  </si>
+  <si>
+    <t>SNU slides, Biological Wastewater Treatment Processes (file 10649)</t>
+  </si>
+  <si>
+    <t>Primary retention time (~2 h), SS (~60%) and BOD (~35%) removal</t>
+  </si>
+  <si>
+    <t>1.47 BODu/BOD5 (proxy for bCOD/BOD5), 4.33 g O₂/g</t>
+  </si>
+  <si>
+    <t>Plant energy: 28 target, 44 guide, 86 observed average (Australia)</t>
   </si>
 </sst>
 </file>
@@ -781,7 +984,7 @@
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -806,6 +1009,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -824,10 +1035,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -863,11 +1075,34 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="13">
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -913,7 +1148,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E011882-5DEB-40AE-A890-C0F7596B9438}" name="Table1" displayName="Table1" ref="A8:E22" totalsRowShown="0" headerRowDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E011882-5DEB-40AE-A890-C0F7596B9438}" name="Table1" displayName="Table1" ref="A8:E22" totalsRowShown="0" headerRowDxfId="12">
   <autoFilter ref="A8:E22" xr:uid="{2E011882-5DEB-40AE-A890-C0F7596B9438}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{2CFF8964-333B-41B4-B18E-46667A53AAB1}" name="Item"/>
@@ -931,10 +1166,10 @@
   <autoFilter ref="A25:E47" xr:uid="{10220E0A-F588-4EEC-850B-7E1E2D028A41}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{A1F7691C-638B-4B2A-B87A-F15E20AFA8EB}" name="Item"/>
-    <tableColumn id="2" xr3:uid="{1CD2E7D3-4A29-4294-A4B7-8E9D80737189}" name="Value" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{DA10D8A3-F7B5-4974-AEA0-6F8A2B592C26}" name="Unit" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{04AE792B-44D8-48DF-B396-C0B22157B224}" name="Status" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{9D8EB251-4103-49AC-B5D7-844043A24FDC}" name="Source" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{1CD2E7D3-4A29-4294-A4B7-8E9D80737189}" name="Value" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{DA10D8A3-F7B5-4974-AEA0-6F8A2B592C26}" name="Unit" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{04AE792B-44D8-48DF-B396-C0B22157B224}" name="Status" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{9D8EB251-4103-49AC-B5D7-844043A24FDC}" name="Source" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -945,10 +1180,24 @@
   <autoFilter ref="A56:E68" xr:uid="{B6766CDA-76F9-4B7B-9856-32898855FE7B}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{E0CFC413-A1FA-4747-9B82-F17D183B11D4}" name="Item"/>
-    <tableColumn id="2" xr3:uid="{55FA7182-7794-4DEB-86DE-BEEF2880D08B}" name="Value" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{B12F1A64-7555-463C-B711-5C7C438C3C74}" name="Unit" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{258BFD5C-E2FB-4A9A-BF30-E43CE2E1A031}" name="Status" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{84CE2C52-D72B-470E-8872-B014E10B2DDE}" name="Source" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{55FA7182-7794-4DEB-86DE-BEEF2880D08B}" name="Value" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{B12F1A64-7555-463C-B711-5C7C438C3C74}" name="Unit" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{258BFD5C-E2FB-4A9A-BF30-E43CE2E1A031}" name="Status" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{84CE2C52-D72B-470E-8872-B014E10B2DDE}" name="Source" dataDxfId="4"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0522E9C3-EAD1-431E-9699-169EBF504702}" name="Table4" displayName="Table4" ref="H8:L24" totalsRowShown="0">
+  <autoFilter ref="H8:L24" xr:uid="{0522E9C3-EAD1-431E-9699-169EBF504702}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{8DE43E2B-D23E-47BE-BA98-E568CE04B603}" name="Item"/>
+    <tableColumn id="2" xr3:uid="{B9E0B95C-7DE8-4D3D-A286-E82B0F44CDB0}" name="Value" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{F941578C-974C-49AC-AFF7-03E35E66ACCB}" name="Unit" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{44D70D08-460E-433A-B6AF-00E5420A8E83}" name="Status" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{A1A93FE9-2B4A-4857-8E44-51CD5214A2EE}" name="Source" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1319,7 +1568,7 @@
         <v>50000</v>
       </c>
       <c r="D5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E5" t="s">
         <v>32</v>
@@ -1336,7 +1585,7 @@
         <v>60</v>
       </c>
       <c r="D6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E6" t="s">
         <v>33</v>
@@ -1353,7 +1602,7 @@
         <v>150</v>
       </c>
       <c r="D7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E7" t="s">
         <v>34</v>
@@ -1370,7 +1619,7 @@
         <v>50</v>
       </c>
       <c r="D8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E8" t="s">
         <v>35</v>
@@ -1387,7 +1636,7 @@
         <v>75</v>
       </c>
       <c r="D9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E9" t="s">
         <v>36</v>
@@ -1404,7 +1653,7 @@
         <v>8</v>
       </c>
       <c r="D10" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E10" t="s">
         <v>37</v>
@@ -1421,10 +1670,10 @@
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E11" t="s">
-        <v>38</v>
+        <v>248</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -1441,7 +1690,7 @@
         <v>26</v>
       </c>
       <c r="E12" t="s">
-        <v>39</v>
+        <v>249</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -1458,7 +1707,7 @@
         <v>26</v>
       </c>
       <c r="E13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -1472,10 +1721,10 @@
         <v>0</v>
       </c>
       <c r="D14" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E14" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -1489,10 +1738,10 @@
         <v>10</v>
       </c>
       <c r="D15" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E15" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -1506,10 +1755,10 @@
         <v>20</v>
       </c>
       <c r="D16" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E16" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -1528,10 +1777,10 @@
         <v>25</v>
       </c>
       <c r="D18" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E18" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -1545,10 +1794,10 @@
         <v>125</v>
       </c>
       <c r="D19" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E19" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -1562,10 +1811,10 @@
         <v>35</v>
       </c>
       <c r="D20" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E20" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -1579,10 +1828,10 @@
         <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E21" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
@@ -1592,269 +1841,269 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C24">
         <f>C7+C8</f>
         <v>200</v>
       </c>
       <c r="D24" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C25" s="2">
         <f>C5*(C7+C8)/1000+C14</f>
         <v>10000</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="26" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C26" s="3">
         <f>C25/24</f>
         <v>416.66666666666669</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="27" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C27" s="4">
         <f>C25/86400</f>
         <v>0.11574074074074074</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C28" s="2">
         <f>C13*C5*C7/1000+C5*C8/1000+C13*C14</f>
         <v>25000</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C29" s="3">
         <f>C28/24</f>
         <v>1041.6666666666667</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="30" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C30" s="4">
         <f>C28/86400</f>
         <v>0.28935185185185186</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="31" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C31" s="2">
         <f>C5*C6/1000</f>
         <v>3000</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C32">
         <f>C31*1000/C25</f>
         <v>300</v>
       </c>
       <c r="D32" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E32" s="4"/>
     </row>
     <row r="33" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C33" s="2">
         <f>C5*C9/1000</f>
         <v>3750</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="34" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C34" s="5">
         <f>C33*1000/C25</f>
         <v>375</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="35" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C35" s="2">
         <f>C5*C10/1000</f>
         <v>400</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="36" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C36" s="2">
         <f>C5*(C10+C11)/1000</f>
         <v>650</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E36" s="5"/>
     </row>
     <row r="37" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C37" s="5">
         <f>C36*1000/C25</f>
         <v>65</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="38" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A38" s="5" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C38" s="5">
         <f>C35*1000/C25</f>
         <v>40</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E38" s="6"/>
     </row>
     <row r="39" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C39" s="5">
         <f>C32*C12</f>
         <v>600</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="40" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C40" s="2">
         <f>C39*C25/1000</f>
         <v>6000</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="41" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A41" s="6" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C41" s="6">
         <f>(1-C18/C32)</f>
         <v>0.91666666666666663</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="42" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" s="6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C42" s="6">
         <f>(1-C19/C39)</f>
         <v>0.79166666666666663</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="43" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A43" s="6" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C43" s="6">
         <f>(1-C20/C34)</f>
         <v>0.90666666666666662</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="44" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A44" s="6" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C44" s="6">
         <f>(1-C21/C38)</f>
         <v>0.875</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="46" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C46" s="2">
         <f>C25*C32/1000-C31</f>
         <v>0</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.35">
@@ -1870,51 +2119,58 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4ED35503-1FDB-4344-A7E4-2522F6B534CB}">
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:L75"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="43.90625" customWidth="1"/>
     <col min="3" max="3" width="11.26953125" customWidth="1"/>
     <col min="4" max="4" width="20.453125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="32.36328125" customWidth="1"/>
+    <col min="8" max="8" width="38.1796875" customWidth="1"/>
+    <col min="9" max="9" width="12.6328125" customWidth="1"/>
+    <col min="11" max="11" width="20.1796875" customWidth="1"/>
+    <col min="12" max="12" width="13.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="11" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="11" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="11" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="11" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A2" s="11" t="s">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A6" s="8"/>
+    </row>
+    <row r="7" spans="1:12" s="8" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="16" t="s">
+        <v>174</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A8" s="7" t="s">
         <v>82</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="11" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="11" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="11" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="8"/>
-    </row>
-    <row r="7" spans="1:5" s="8" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="16" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="7" t="s">
-        <v>86</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>2</v>
@@ -1923,258 +2179,515 @@
         <v>3</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+        <v>84</v>
+      </c>
+      <c r="H8" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="I8" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="J8" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="K8" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="L8" s="13" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B9">
         <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D9" t="s">
-        <v>91</v>
+        <v>251</v>
       </c>
       <c r="E9" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+        <v>26</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="I9" s="10">
+        <v>5</v>
+      </c>
+      <c r="J9" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="L9" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B10" s="10">
         <v>100</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>128</v>
+        <v>251</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+        <v>26</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="I10" s="10">
+        <v>0.3</v>
+      </c>
+      <c r="J10" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="K10" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="L10" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="58" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B11" s="10">
         <v>2</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>131</v>
+        <v>285</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+        <v>286</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="I11" s="10">
+        <v>6</v>
+      </c>
+      <c r="J11" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="K11" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="L11" s="10" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B12" s="10">
         <v>30</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>96</v>
+        <v>287</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+        <v>288</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="I12" s="10">
+        <v>0.9</v>
+      </c>
+      <c r="J12" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="K12" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="L12" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="58" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="B13" s="10">
         <v>60</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>99</v>
+        <v>289</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+        <v>288</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="I13" s="10">
+        <v>0.8</v>
+      </c>
+      <c r="J13" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="K13" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="L13" s="10" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="10" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="B14" s="10">
         <v>30</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+        <v>93</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="I14" s="10">
+        <v>0.92</v>
+      </c>
+      <c r="J14" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="K14" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="L14" s="10" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="B15" s="10">
         <v>10</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+        <v>93</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="I15" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="J15" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="K15" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="L15" s="10" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B16" s="10">
         <v>0</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+        <v>93</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="I16" s="10" t="s">
+        <v>224</v>
+      </c>
+      <c r="J16" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="K16" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="L16" s="10" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="B17" s="10">
         <v>2</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+        <v>93</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="I17" s="10">
+        <v>2</v>
+      </c>
+      <c r="J17" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="K17" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="L17" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="B18" s="10">
         <v>0.9</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+        <v>103</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="I18" s="10">
+        <v>0.27900000000000003</v>
+      </c>
+      <c r="J18" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="K18" s="10" t="s">
+        <v>228</v>
+      </c>
+      <c r="L18" s="10" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="10" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="B19" s="10">
         <v>20</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+        <v>107</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="I19" s="10">
+        <v>1.4</v>
+      </c>
+      <c r="J19" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="K19" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="L19" s="10" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="10" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="B20" s="10">
         <v>10</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+        <v>107</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="I20" s="10">
+        <v>0.6</v>
+      </c>
+      <c r="J20" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="K20" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="L20" s="10" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="10" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+        <v>107</v>
+      </c>
+      <c r="H21" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="I21" s="10">
+        <v>10</v>
+      </c>
+      <c r="J21" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="K21" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="L21" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A22" s="10" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="B22" s="10">
         <v>180</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>105</v>
+        <v>251</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" s="12" customFormat="1" x14ac:dyDescent="0.35">
+        <v>26</v>
+      </c>
+      <c r="H22" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="I22" s="15">
+        <v>8760</v>
+      </c>
+      <c r="J22" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="K22" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="L22" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="H23" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="I23" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="J23" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="K23" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="L23" s="10" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" s="12" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A24" s="12" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+        <v>173</v>
+      </c>
+      <c r="H24" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="I24" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="J24" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="K24" s="10" t="s">
+        <v>294</v>
+      </c>
+      <c r="L24" s="10" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A25" s="13" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B25" s="13" t="s">
         <v>2</v>
@@ -2183,429 +2696,447 @@
         <v>3</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="10" t="s">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="B26" s="10">
         <v>10</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+        <v>93</v>
+      </c>
+      <c r="H26" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="10" t="s">
-        <v>135</v>
+        <v>120</v>
       </c>
       <c r="B27" s="10">
         <v>0.5</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>136</v>
+        <v>121</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+        <v>123</v>
+      </c>
+      <c r="H27" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="10" t="s">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+      <c r="H28" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A29" s="10" t="s">
-        <v>142</v>
+        <v>127</v>
       </c>
       <c r="B29" s="10">
         <v>2</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>143</v>
+        <v>128</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+      <c r="H29" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A30" s="10" t="s">
-        <v>144</v>
+        <v>129</v>
       </c>
       <c r="B30" s="10">
         <v>1.3</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+      <c r="H30" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A31" s="10" t="s">
-        <v>145</v>
+        <v>130</v>
       </c>
       <c r="B31" s="10">
         <v>2</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+      <c r="H31" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" ht="58" x14ac:dyDescent="0.35">
       <c r="A32" s="10" t="s">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="B32" s="10">
         <v>1</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A33" s="10" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>151</v>
+        <v>290</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A34" s="10" t="s">
-        <v>152</v>
+        <v>136</v>
       </c>
       <c r="B34" s="10">
         <v>1.47</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>154</v>
+        <v>291</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>155</v>
+        <v>139</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
       <c r="B35" s="10">
         <v>5</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A36" s="10" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
       <c r="B36" s="10">
         <v>0.45</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A37" s="10" t="s">
-        <v>161</v>
+        <v>145</v>
       </c>
       <c r="B37" s="10">
         <v>0.1</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>136</v>
+        <v>121</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>162</v>
+        <v>146</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A38" s="10" t="s">
-        <v>164</v>
+        <v>148</v>
       </c>
       <c r="B38" s="10">
         <v>1.04</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>165</v>
+        <v>149</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>166</v>
+        <v>150</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A39" s="10" t="s">
-        <v>167</v>
+        <v>151</v>
       </c>
       <c r="B39" s="10">
         <v>0.15</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>168</v>
+        <v>152</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="10" t="s">
-        <v>169</v>
+        <v>153</v>
       </c>
       <c r="B40" s="10">
         <v>0.85</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>170</v>
+        <v>251</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>171</v>
+        <v>26</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A41" s="10" t="s">
-        <v>172</v>
+        <v>154</v>
       </c>
       <c r="B41" s="15">
         <v>4000</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>173</v>
+        <v>155</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>174</v>
+        <v>156</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="10" t="s">
-        <v>175</v>
+        <v>157</v>
       </c>
       <c r="B42" s="10">
         <v>0.75</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="10" t="s">
-        <v>176</v>
+        <v>158</v>
       </c>
       <c r="B43" s="10">
         <v>0.4</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A44" s="10" t="s">
-        <v>177</v>
+        <v>159</v>
       </c>
       <c r="B44" s="10">
         <v>0.124</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>179</v>
+        <v>161</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="10" t="s">
-        <v>180</v>
+        <v>162</v>
       </c>
       <c r="B45" s="10">
         <v>1.42</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>154</v>
+        <v>138</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="10" t="s">
-        <v>181</v>
+        <v>163</v>
       </c>
       <c r="B46" s="10">
         <v>4.33</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>154</v>
+        <v>138</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>182</v>
+        <v>164</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A47" s="10" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="B47" s="10">
         <v>7.14</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>184</v>
+        <v>166</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>185</v>
+        <v>167</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="7" t="s">
-        <v>186</v>
+        <v>168</v>
       </c>
       <c r="B49" s="7"/>
       <c r="C49" s="7"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="7" t="s">
-        <v>187</v>
+        <v>169</v>
       </c>
       <c r="B50" s="7"/>
       <c r="C50" s="7"/>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="7" t="s">
-        <v>188</v>
+        <v>170</v>
       </c>
       <c r="B51" s="7"/>
       <c r="C51" s="7"/>
     </row>
     <row r="52" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A52" s="7" t="s">
-        <v>189</v>
+        <v>292</v>
       </c>
       <c r="B52" s="7"/>
       <c r="C52" s="7"/>
     </row>
     <row r="53" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A53" s="7" t="s">
-        <v>190</v>
+        <v>171</v>
       </c>
       <c r="B53" s="7"/>
       <c r="C53" s="7"/>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
-        <v>191</v>
+        <v>172</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="13" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B56" s="13" t="s">
         <v>2</v>
@@ -2614,219 +3145,219 @@
         <v>3</v>
       </c>
       <c r="D56" s="13" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E56" s="13" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="10" t="s">
-        <v>194</v>
+        <v>175</v>
       </c>
       <c r="B57" s="10">
         <v>100</v>
       </c>
       <c r="C57" s="10" t="s">
-        <v>195</v>
+        <v>176</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>196</v>
+        <v>99</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A58" s="10" t="s">
-        <v>198</v>
+        <v>177</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>199</v>
+        <v>178</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D58" s="10" t="s">
-        <v>200</v>
+        <v>293</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>141</v>
+        <v>26</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A59" s="10" t="s">
-        <v>201</v>
+        <v>179</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>202</v>
+        <v>180</v>
       </c>
       <c r="C59" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="D59" s="10" t="s">
-        <v>203</v>
+        <v>181</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>141</v>
+        <v>26</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A60" s="10" t="s">
-        <v>204</v>
+        <v>182</v>
       </c>
       <c r="B60" s="10">
         <v>24</v>
       </c>
       <c r="C60" s="10" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="D60" s="10" t="s">
-        <v>205</v>
+        <v>183</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>206</v>
+        <v>184</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A61" s="10" t="s">
-        <v>207</v>
+        <v>185</v>
       </c>
       <c r="B61" s="10">
         <v>44</v>
       </c>
       <c r="C61" s="10" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="D61" s="10" t="s">
-        <v>208</v>
+        <v>186</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="10" t="s">
-        <v>209</v>
+        <v>187</v>
       </c>
       <c r="B62" s="10">
         <v>144</v>
       </c>
       <c r="C62" s="10" t="s">
-        <v>210</v>
+        <v>188</v>
       </c>
       <c r="D62" s="10" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
       <c r="E62" s="10" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="10" t="s">
-        <v>211</v>
+        <v>189</v>
       </c>
       <c r="B63" s="10">
         <v>216</v>
       </c>
       <c r="C63" s="10" t="s">
-        <v>210</v>
+        <v>188</v>
       </c>
       <c r="D63" s="10" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A64" s="10" t="s">
-        <v>212</v>
+        <v>190</v>
       </c>
       <c r="B64" s="10">
         <v>375</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>213</v>
+        <v>191</v>
       </c>
       <c r="D64" s="10" t="s">
-        <v>214</v>
+        <v>252</v>
       </c>
       <c r="E64" s="10" t="s">
-        <v>215</v>
+        <v>26</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A65" s="10" t="s">
-        <v>216</v>
+        <v>192</v>
       </c>
       <c r="B65" s="10">
         <v>2</v>
       </c>
       <c r="C65" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="D65" s="10" t="s">
-        <v>217</v>
+        <v>193</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>218</v>
+        <v>26</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A66" s="10" t="s">
-        <v>219</v>
+        <v>194</v>
       </c>
       <c r="B66" s="10">
         <v>4</v>
       </c>
       <c r="C66" s="10" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="D66" s="10" t="s">
-        <v>220</v>
+        <v>195</v>
       </c>
       <c r="E66" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="58" x14ac:dyDescent="0.35">
       <c r="A67" s="10" t="s">
-        <v>221</v>
+        <v>196</v>
       </c>
       <c r="B67" s="10" t="s">
-        <v>222</v>
+        <v>197</v>
       </c>
       <c r="C67" s="10" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D67" s="10" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A68" s="10" t="s">
-        <v>223</v>
+        <v>198</v>
       </c>
       <c r="B68" s="10" t="s">
-        <v>224</v>
+        <v>199</v>
       </c>
       <c r="C68" s="10" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="D68" s="10" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A70" s="7" t="s">
-        <v>225</v>
+        <v>200</v>
       </c>
       <c r="B70" s="7"/>
       <c r="C70" s="7"/>
@@ -2834,7 +3365,7 @@
     </row>
     <row r="71" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A71" s="7" t="s">
-        <v>226</v>
+        <v>201</v>
       </c>
       <c r="B71" s="7"/>
       <c r="C71" s="7"/>
@@ -2842,7 +3373,7 @@
     </row>
     <row r="72" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A72" s="7" t="s">
-        <v>227</v>
+        <v>202</v>
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="7"/>
@@ -2850,7 +3381,7 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="7" t="s">
-        <v>228</v>
+        <v>203</v>
       </c>
       <c r="B73" s="7"/>
       <c r="C73" s="7"/>
@@ -2858,7 +3389,7 @@
     </row>
     <row r="74" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A74" s="7" t="s">
-        <v>229</v>
+        <v>204</v>
       </c>
       <c r="B74" s="7"/>
       <c r="C74" s="7"/>
@@ -2866,7 +3397,7 @@
     </row>
     <row r="75" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A75" s="7" t="s">
-        <v>230</v>
+        <v>205</v>
       </c>
       <c r="B75" s="7"/>
       <c r="C75" s="7"/>
@@ -2874,10 +3405,243 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="3">
+  <tableParts count="4">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77CC8B4D-B4FF-4676-9E1B-DF5D2CBAA55E}">
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="3.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.1796875" customWidth="1"/>
+    <col min="3" max="3" width="37.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="17" t="s">
+        <v>254</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>255</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="18">
+        <v>1</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>256</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>257</v>
+      </c>
+      <c r="D2" s="20" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="18">
+        <v>2</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>258</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>259</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="18">
+        <v>3</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>260</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>261</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" s="18">
+        <v>4</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>295</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>296</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="18">
+        <v>5</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>262</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>263</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="18">
+        <v>6</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>264</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8" s="18">
+        <v>7</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>164</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>297</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="18">
+        <v>8</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>265</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>266</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="18">
+        <v>9</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>184</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>267</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A11" s="18">
+        <v>10</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A12" s="18">
+        <v>11</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>269</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" s="18">
+        <v>12</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>213</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>270</v>
+      </c>
+      <c r="D13" s="20" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" s="18">
+        <v>13</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>242</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>298</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="19"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{29ABE9EA-56CB-4E87-850C-CE12B10FE191}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{99535719-D2EF-4A5F-B8CC-BE9175C46BF5}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{12B8C91F-094F-4ACC-9CE0-02B1BA4BE38F}"/>
+    <hyperlink ref="D6" r:id="rId4" xr:uid="{C290A0CE-7C5F-453C-BE44-B6F04397C67E}"/>
+    <hyperlink ref="D5" r:id="rId5" xr:uid="{F2AB4DB8-62BB-4A0A-BF1E-CD309AFDB86F}"/>
+    <hyperlink ref="D7" r:id="rId6" xr:uid="{C138734D-6565-4F4E-AAD5-746926ECBC04}"/>
+    <hyperlink ref="D8" r:id="rId7" xr:uid="{211A5539-A811-41D2-A1B4-C3EA4D49C84F}"/>
+    <hyperlink ref="D9" r:id="rId8" xr:uid="{62C25677-63B3-4578-B908-7ED00A16A934}"/>
+    <hyperlink ref="D10" r:id="rId9" xr:uid="{5F171C21-2F40-4CFF-BFBA-47ED8E8B3428}"/>
+    <hyperlink ref="D11" r:id="rId10" xr:uid="{1C26169E-AD44-4651-8420-7C5A92947B1E}"/>
+    <hyperlink ref="D12" r:id="rId11" xr:uid="{DE30D3E2-114F-4554-A542-63476B43E3B5}"/>
+    <hyperlink ref="D13" r:id="rId12" xr:uid="{78CCA610-ABFB-4498-8654-B164D85FBA37}"/>
+    <hyperlink ref="D14" r:id="rId13" xr:uid="{DF0370B4-4C65-4B88-83E8-9D227D3BFAE9}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId14"/>
+</worksheet>
 </file>
</xml_diff>